<commit_message>
NIS2 preview: close review items 5.2 and 13.ε (remove unrelated article link)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M4snhbgdNH6z5QRgt779xt
</commit_message>
<xml_diff>
--- a/static/downloads/nis2-kya-1689-2025-microsoft-365-checklist.xlsx
+++ b/static/downloads/nis2-kya-1689-2025-microsoft-365-checklist.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="947" uniqueCount="560">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="559">
   <si>
     <t xml:space="preserve">ΚΥΑ 1689/2025 και Microsoft 365: checklist συμμόρφωσης</t>
   </si>
@@ -728,9 +728,6 @@
   </si>
   <si>
     <t xml:space="preserve">Microsoft Entra ID Governance (lifecycle workflows)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://thecybersec.gr/posts/new-features/defender-xdr-unified-response-actions-identity-accounts/</t>
   </si>
   <si>
     <t xml:space="preserve">13.στ</t>
@@ -3892,9 +3889,7 @@
         <v>228</v>
       </c>
       <c r="J41" s="8"/>
-      <c r="K41" s="8" t="s">
-        <v>229</v>
-      </c>
+      <c r="K41" s="8"/>
       <c r="L41" s="9"/>
       <c r="M41" s="10"/>
       <c r="N41" s="10"/>
@@ -3903,7 +3898,7 @@
     </row>
     <row r="42" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B42" s="7" t="n">
         <v>13</v>
@@ -3915,21 +3910,21 @@
         <v>45</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F42" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G42" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="H42" s="8" t="s">
         <v>232</v>
-      </c>
-      <c r="H42" s="8" t="s">
-        <v>233</v>
       </c>
       <c r="I42" s="8"/>
       <c r="J42" s="8"/>
       <c r="K42" s="8" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="L42" s="9"/>
       <c r="M42" s="10"/>
@@ -3939,7 +3934,7 @@
     </row>
     <row r="43" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B43" s="7" t="n">
         <v>13</v>
@@ -3951,21 +3946,21 @@
         <v>45</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F43" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G43" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="H43" s="8" t="s">
         <v>237</v>
-      </c>
-      <c r="H43" s="8" t="s">
-        <v>238</v>
       </c>
       <c r="I43" s="8"/>
       <c r="J43" s="8"/>
       <c r="K43" s="8" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="L43" s="9"/>
       <c r="M43" s="10"/>
@@ -3975,7 +3970,7 @@
     </row>
     <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B44" s="7" t="n">
         <v>13</v>
@@ -3987,19 +3982,19 @@
         <v>45</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F44" s="8" t="s">
         <v>23</v>
       </c>
       <c r="G44" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="H44" s="8" t="s">
         <v>242</v>
       </c>
-      <c r="H44" s="8" t="s">
+      <c r="I44" s="8" t="s">
         <v>243</v>
-      </c>
-      <c r="I44" s="8" t="s">
-        <v>244</v>
       </c>
       <c r="J44" s="8"/>
       <c r="K44" s="8" t="s">
@@ -4013,33 +4008,33 @@
     </row>
     <row r="45" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B45" s="7" t="n">
         <v>14</v>
       </c>
       <c r="C45" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="D45" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E45" s="8" t="s">
         <v>246</v>
-      </c>
-      <c r="D45" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="E45" s="8" t="s">
-        <v>247</v>
       </c>
       <c r="F45" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G45" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="H45" s="8" t="s">
         <v>248</v>
-      </c>
-      <c r="H45" s="8" t="s">
-        <v>249</v>
       </c>
       <c r="I45" s="8"/>
       <c r="J45" s="8"/>
       <c r="K45" s="8" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="L45" s="9"/>
       <c r="M45" s="10"/>
@@ -4049,35 +4044,35 @@
     </row>
     <row r="46" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B46" s="7" t="n">
         <v>14</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D46" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F46" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G46" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="H46" s="8" t="s">
         <v>253</v>
       </c>
-      <c r="H46" s="8" t="s">
+      <c r="I46" s="8" t="s">
         <v>254</v>
-      </c>
-      <c r="I46" s="8" t="s">
-        <v>255</v>
       </c>
       <c r="J46" s="8"/>
       <c r="K46" s="8" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="L46" s="9"/>
       <c r="M46" s="10"/>
@@ -4087,35 +4082,35 @@
     </row>
     <row r="47" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B47" s="7" t="n">
         <v>14</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D47" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F47" s="8" t="s">
         <v>23</v>
       </c>
       <c r="G47" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="H47" s="8" t="s">
         <v>259</v>
-      </c>
-      <c r="H47" s="8" t="s">
-        <v>260</v>
       </c>
       <c r="I47" s="8"/>
       <c r="J47" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="K47" s="8" t="s">
         <v>261</v>
-      </c>
-      <c r="K47" s="8" t="s">
-        <v>262</v>
       </c>
       <c r="L47" s="9"/>
       <c r="M47" s="10"/>
@@ -4125,28 +4120,28 @@
     </row>
     <row r="48" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B48" s="7" t="n">
         <v>14</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D48" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F48" s="8" t="s">
         <v>23</v>
       </c>
       <c r="G48" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="H48" s="8" t="s">
         <v>265</v>
-      </c>
-      <c r="H48" s="8" t="s">
-        <v>266</v>
       </c>
       <c r="I48" s="8"/>
       <c r="J48" s="8"/>
@@ -4161,28 +4156,28 @@
     </row>
     <row r="49" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B49" s="7" t="n">
         <v>15</v>
       </c>
       <c r="C49" s="8" t="s">
+        <v>267</v>
+      </c>
+      <c r="D49" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E49" s="8" t="s">
         <v>268</v>
-      </c>
-      <c r="D49" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="E49" s="8" t="s">
-        <v>269</v>
       </c>
       <c r="F49" s="8" t="s">
         <v>25</v>
       </c>
       <c r="G49" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="H49" s="8" t="s">
         <v>270</v>
-      </c>
-      <c r="H49" s="8" t="s">
-        <v>271</v>
       </c>
       <c r="I49" s="8"/>
       <c r="J49" s="8"/>
@@ -4195,35 +4190,35 @@
     </row>
     <row r="50" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B50" s="7" t="n">
         <v>15</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D50" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F50" s="8" t="s">
         <v>25</v>
       </c>
       <c r="G50" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="H50" s="8" t="s">
         <v>274</v>
       </c>
-      <c r="H50" s="8" t="s">
+      <c r="I50" s="8" t="s">
         <v>275</v>
-      </c>
-      <c r="I50" s="8" t="s">
-        <v>276</v>
       </c>
       <c r="J50" s="8"/>
       <c r="K50" s="8" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="L50" s="9"/>
       <c r="M50" s="10"/>
@@ -4233,31 +4228,31 @@
     </row>
     <row r="51" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B51" s="7" t="n">
         <v>15</v>
       </c>
       <c r="C51" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D51" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F51" s="8" t="s">
         <v>25</v>
       </c>
       <c r="G51" s="8" t="s">
+        <v>279</v>
+      </c>
+      <c r="H51" s="8" t="s">
         <v>280</v>
       </c>
-      <c r="H51" s="8" t="s">
+      <c r="I51" s="8" t="s">
         <v>281</v>
-      </c>
-      <c r="I51" s="8" t="s">
-        <v>282</v>
       </c>
       <c r="J51" s="8"/>
       <c r="K51" s="8"/>
@@ -4269,31 +4264,31 @@
     </row>
     <row r="52" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B52" s="7" t="n">
         <v>15</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D52" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E52" s="8" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F52" s="8" t="s">
         <v>25</v>
       </c>
       <c r="G52" s="8" t="s">
+        <v>284</v>
+      </c>
+      <c r="H52" s="8" t="s">
         <v>285</v>
       </c>
-      <c r="H52" s="8" t="s">
+      <c r="I52" s="8" t="s">
         <v>286</v>
-      </c>
-      <c r="I52" s="8" t="s">
-        <v>287</v>
       </c>
       <c r="J52" s="8"/>
       <c r="K52" s="8"/>
@@ -4305,33 +4300,33 @@
     </row>
     <row r="53" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B53" s="7" t="n">
         <v>16</v>
       </c>
       <c r="C53" s="8" t="s">
+        <v>288</v>
+      </c>
+      <c r="D53" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E53" s="8" t="s">
         <v>289</v>
-      </c>
-      <c r="D53" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="E53" s="8" t="s">
-        <v>290</v>
       </c>
       <c r="F53" s="8" t="s">
         <v>23</v>
       </c>
       <c r="G53" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="H53" s="8" t="s">
         <v>291</v>
-      </c>
-      <c r="H53" s="8" t="s">
-        <v>292</v>
       </c>
       <c r="I53" s="8"/>
       <c r="J53" s="8"/>
       <c r="K53" s="8" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="L53" s="9"/>
       <c r="M53" s="10"/>
@@ -4341,19 +4336,19 @@
     </row>
     <row r="54" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B54" s="7" t="n">
         <v>16</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D54" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E54" s="8" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F54" s="8" t="s">
         <v>25</v>
@@ -4375,33 +4370,33 @@
     </row>
     <row r="55" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B55" s="7" t="n">
         <v>17</v>
       </c>
       <c r="C55" s="8" t="s">
+        <v>296</v>
+      </c>
+      <c r="D55" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E55" s="8" t="s">
         <v>297</v>
-      </c>
-      <c r="D55" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="E55" s="8" t="s">
-        <v>298</v>
       </c>
       <c r="F55" s="8" t="s">
         <v>23</v>
       </c>
       <c r="G55" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="H55" s="8" t="s">
         <v>299</v>
-      </c>
-      <c r="H55" s="8" t="s">
-        <v>300</v>
       </c>
       <c r="I55" s="8"/>
       <c r="J55" s="8"/>
       <c r="K55" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="L55" s="9"/>
       <c r="M55" s="10"/>
@@ -4411,33 +4406,33 @@
     </row>
     <row r="56" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B56" s="7" t="n">
         <v>17</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D56" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F56" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G56" s="8" t="s">
+        <v>303</v>
+      </c>
+      <c r="H56" s="8" t="s">
         <v>304</v>
-      </c>
-      <c r="H56" s="8" t="s">
-        <v>305</v>
       </c>
       <c r="I56" s="8"/>
       <c r="J56" s="8"/>
       <c r="K56" s="8" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="L56" s="9"/>
       <c r="M56" s="10"/>
@@ -4447,33 +4442,33 @@
     </row>
     <row r="57" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B57" s="7" t="n">
         <v>17</v>
       </c>
       <c r="C57" s="8" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D57" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F57" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G57" s="8" t="s">
+        <v>308</v>
+      </c>
+      <c r="H57" s="8" t="s">
         <v>309</v>
-      </c>
-      <c r="H57" s="8" t="s">
-        <v>310</v>
       </c>
       <c r="I57" s="8"/>
       <c r="J57" s="8"/>
       <c r="K57" s="8" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="L57" s="9"/>
       <c r="M57" s="10"/>
@@ -4483,33 +4478,33 @@
     </row>
     <row r="58" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B58" s="7" t="n">
         <v>17</v>
       </c>
       <c r="C58" s="8" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D58" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E58" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="F58" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G58" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="H58" s="8" t="s">
         <v>314</v>
-      </c>
-      <c r="H58" s="8" t="s">
-        <v>315</v>
       </c>
       <c r="I58" s="8"/>
       <c r="J58" s="8"/>
       <c r="K58" s="8" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="L58" s="9"/>
       <c r="M58" s="10"/>
@@ -4519,37 +4514,37 @@
     </row>
     <row r="59" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B59" s="7" t="n">
         <v>17</v>
       </c>
       <c r="C59" s="8" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D59" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F59" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G59" s="8" t="s">
+        <v>318</v>
+      </c>
+      <c r="H59" s="8" t="s">
         <v>319</v>
       </c>
-      <c r="H59" s="8" t="s">
+      <c r="I59" s="8" t="s">
         <v>320</v>
       </c>
-      <c r="I59" s="8" t="s">
+      <c r="J59" s="8" t="s">
         <v>321</v>
       </c>
-      <c r="J59" s="8" t="s">
-        <v>322</v>
-      </c>
       <c r="K59" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="L59" s="9"/>
       <c r="M59" s="10"/>
@@ -4559,33 +4554,33 @@
     </row>
     <row r="60" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B60" s="7" t="n">
         <v>17</v>
       </c>
       <c r="C60" s="8" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D60" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E60" s="8" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="F60" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G60" s="8" t="s">
+        <v>324</v>
+      </c>
+      <c r="H60" s="8" t="s">
         <v>325</v>
-      </c>
-      <c r="H60" s="8" t="s">
-        <v>326</v>
       </c>
       <c r="I60" s="8"/>
       <c r="J60" s="8"/>
       <c r="K60" s="8" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="L60" s="9"/>
       <c r="M60" s="10"/>
@@ -4595,19 +4590,19 @@
     </row>
     <row r="61" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B61" s="7" t="n">
         <v>17</v>
       </c>
       <c r="C61" s="8" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D61" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E61" s="8" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F61" s="8" t="s">
         <v>25</v>
@@ -4616,7 +4611,7 @@
         <v>92</v>
       </c>
       <c r="H61" s="8" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="I61" s="8"/>
       <c r="J61" s="8"/>
@@ -4629,19 +4624,19 @@
     </row>
     <row r="62" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B62" s="7" t="n">
         <v>18</v>
       </c>
       <c r="C62" s="8" t="s">
+        <v>331</v>
+      </c>
+      <c r="D62" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E62" s="8" t="s">
         <v>332</v>
-      </c>
-      <c r="D62" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="E62" s="8" t="s">
-        <v>333</v>
       </c>
       <c r="F62" s="8" t="s">
         <v>25</v>
@@ -4650,7 +4645,7 @@
         <v>92</v>
       </c>
       <c r="H62" s="8" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="I62" s="8"/>
       <c r="J62" s="8"/>
@@ -4663,28 +4658,28 @@
     </row>
     <row r="63" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B63" s="7" t="n">
         <v>18</v>
       </c>
       <c r="C63" s="8" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D63" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F63" s="8" t="s">
         <v>25</v>
       </c>
       <c r="G63" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="H63" s="8" t="s">
         <v>337</v>
-      </c>
-      <c r="H63" s="8" t="s">
-        <v>338</v>
       </c>
       <c r="I63" s="8"/>
       <c r="J63" s="8"/>
@@ -4697,28 +4692,28 @@
     </row>
     <row r="64" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B64" s="7" t="n">
         <v>18</v>
       </c>
       <c r="C64" s="8" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D64" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E64" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="F64" s="8" t="s">
         <v>23</v>
       </c>
       <c r="G64" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="H64" s="8" t="s">
         <v>341</v>
-      </c>
-      <c r="H64" s="8" t="s">
-        <v>342</v>
       </c>
       <c r="I64" s="8"/>
       <c r="J64" s="8"/>
@@ -4733,28 +4728,28 @@
     </row>
     <row r="65" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B65" s="7" t="n">
         <v>18</v>
       </c>
       <c r="C65" s="8" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D65" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="F65" s="8" t="s">
         <v>23</v>
       </c>
       <c r="G65" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="H65" s="8" t="s">
         <v>345</v>
-      </c>
-      <c r="H65" s="8" t="s">
-        <v>346</v>
       </c>
       <c r="I65" s="8"/>
       <c r="J65" s="8"/>
@@ -4769,28 +4764,28 @@
     </row>
     <row r="66" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B66" s="7" t="n">
         <v>18</v>
       </c>
       <c r="C66" s="8" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D66" s="8" t="s">
         <v>75</v>
       </c>
       <c r="E66" s="8" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="F66" s="8" t="s">
         <v>25</v>
       </c>
       <c r="G66" s="8" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H66" s="8" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="I66" s="8"/>
       <c r="J66" s="8"/>
@@ -4803,33 +4798,33 @@
     </row>
     <row r="67" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B67" s="7" t="n">
         <v>18</v>
       </c>
       <c r="C67" s="8" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D67" s="8" t="s">
         <v>75</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="F67" s="8" t="s">
         <v>23</v>
       </c>
       <c r="G67" s="8" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H67" s="8" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="I67" s="8"/>
       <c r="J67" s="8"/>
       <c r="K67" s="8" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="L67" s="9"/>
       <c r="M67" s="10"/>
@@ -4839,19 +4834,19 @@
     </row>
     <row r="68" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B68" s="7" t="n">
         <v>19</v>
       </c>
       <c r="C68" s="8" t="s">
+        <v>354</v>
+      </c>
+      <c r="D68" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E68" s="8" t="s">
         <v>355</v>
-      </c>
-      <c r="D68" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="E68" s="8" t="s">
-        <v>356</v>
       </c>
       <c r="F68" s="8" t="s">
         <v>25</v>
@@ -4860,7 +4855,7 @@
         <v>92</v>
       </c>
       <c r="H68" s="8" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="I68" s="8"/>
       <c r="J68" s="8"/>
@@ -4873,35 +4868,35 @@
     </row>
     <row r="69" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B69" s="7" t="n">
         <v>19</v>
       </c>
       <c r="C69" s="8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D69" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E69" s="8" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F69" s="8" t="s">
         <v>23</v>
       </c>
       <c r="G69" s="8" t="s">
+        <v>359</v>
+      </c>
+      <c r="H69" s="8" t="s">
         <v>360</v>
       </c>
-      <c r="H69" s="8" t="s">
+      <c r="I69" s="8" t="s">
         <v>361</v>
-      </c>
-      <c r="I69" s="8" t="s">
-        <v>362</v>
       </c>
       <c r="J69" s="8"/>
       <c r="K69" s="8" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L69" s="9"/>
       <c r="M69" s="10"/>
@@ -4911,33 +4906,33 @@
     </row>
     <row r="70" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B70" s="7" t="n">
         <v>19</v>
       </c>
       <c r="C70" s="8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D70" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E70" s="8" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="F70" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G70" s="8" t="s">
+        <v>365</v>
+      </c>
+      <c r="H70" s="8" t="s">
         <v>366</v>
-      </c>
-      <c r="H70" s="8" t="s">
-        <v>367</v>
       </c>
       <c r="I70" s="8"/>
       <c r="J70" s="8"/>
       <c r="K70" s="8" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="L70" s="9"/>
       <c r="M70" s="10"/>
@@ -4947,28 +4942,28 @@
     </row>
     <row r="71" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B71" s="7" t="n">
         <v>19</v>
       </c>
       <c r="C71" s="8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D71" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E71" s="8" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F71" s="8" t="s">
         <v>23</v>
       </c>
       <c r="G71" s="8" t="s">
+        <v>370</v>
+      </c>
+      <c r="H71" s="8" t="s">
         <v>371</v>
-      </c>
-      <c r="H71" s="8" t="s">
-        <v>372</v>
       </c>
       <c r="I71" s="8"/>
       <c r="J71" s="8"/>
@@ -4983,33 +4978,33 @@
     </row>
     <row r="72" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="7" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B72" s="7" t="n">
         <v>19</v>
       </c>
       <c r="C72" s="8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D72" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E72" s="8" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="F72" s="8" t="s">
         <v>23</v>
       </c>
       <c r="G72" s="8" t="s">
+        <v>374</v>
+      </c>
+      <c r="H72" s="8" t="s">
         <v>375</v>
-      </c>
-      <c r="H72" s="8" t="s">
-        <v>376</v>
       </c>
       <c r="I72" s="8"/>
       <c r="J72" s="8"/>
       <c r="K72" s="8" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="L72" s="9"/>
       <c r="M72" s="10"/>
@@ -5019,28 +5014,28 @@
     </row>
     <row r="73" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="7" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B73" s="7" t="n">
         <v>19</v>
       </c>
       <c r="C73" s="8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D73" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="F73" s="8" t="s">
         <v>25</v>
       </c>
       <c r="G73" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="H73" s="8" t="s">
         <v>380</v>
-      </c>
-      <c r="H73" s="8" t="s">
-        <v>381</v>
       </c>
       <c r="I73" s="8"/>
       <c r="J73" s="8"/>
@@ -5053,33 +5048,33 @@
     </row>
     <row r="74" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="7" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B74" s="7" t="n">
         <v>19</v>
       </c>
       <c r="C74" s="8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D74" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E74" s="8" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="F74" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G74" s="8" t="s">
+        <v>383</v>
+      </c>
+      <c r="H74" s="8" t="s">
         <v>384</v>
-      </c>
-      <c r="H74" s="8" t="s">
-        <v>385</v>
       </c>
       <c r="I74" s="8"/>
       <c r="J74" s="8"/>
       <c r="K74" s="8" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="L74" s="9"/>
       <c r="M74" s="10"/>
@@ -5089,35 +5084,35 @@
     </row>
     <row r="75" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="7" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B75" s="7" t="n">
         <v>19</v>
       </c>
       <c r="C75" s="8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D75" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E75" s="8" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F75" s="8" t="s">
         <v>23</v>
       </c>
       <c r="G75" s="8" t="s">
+        <v>388</v>
+      </c>
+      <c r="H75" s="8" t="s">
         <v>389</v>
-      </c>
-      <c r="H75" s="8" t="s">
-        <v>390</v>
       </c>
       <c r="I75" s="8"/>
       <c r="J75" s="8" t="s">
+        <v>390</v>
+      </c>
+      <c r="K75" s="8" t="s">
         <v>391</v>
-      </c>
-      <c r="K75" s="8" t="s">
-        <v>392</v>
       </c>
       <c r="L75" s="9"/>
       <c r="M75" s="10"/>
@@ -5127,33 +5122,33 @@
     </row>
     <row r="76" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="7" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B76" s="7" t="n">
         <v>19</v>
       </c>
       <c r="C76" s="8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D76" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E76" s="8" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F76" s="8" t="s">
         <v>23</v>
       </c>
       <c r="G76" s="8" t="s">
+        <v>394</v>
+      </c>
+      <c r="H76" s="8" t="s">
         <v>395</v>
-      </c>
-      <c r="H76" s="8" t="s">
-        <v>396</v>
       </c>
       <c r="I76" s="8"/>
       <c r="J76" s="8"/>
       <c r="K76" s="8" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="L76" s="9"/>
       <c r="M76" s="10"/>
@@ -5163,31 +5158,31 @@
     </row>
     <row r="77" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="7" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B77" s="7" t="n">
         <v>19</v>
       </c>
       <c r="C77" s="8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D77" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E77" s="8" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="F77" s="8" t="s">
         <v>25</v>
       </c>
       <c r="G77" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="H77" s="8" t="s">
         <v>400</v>
       </c>
-      <c r="H77" s="8" t="s">
+      <c r="I77" s="8" t="s">
         <v>401</v>
-      </c>
-      <c r="I77" s="8" t="s">
-        <v>402</v>
       </c>
       <c r="J77" s="8"/>
       <c r="K77" s="8"/>
@@ -5199,19 +5194,19 @@
     </row>
     <row r="78" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="7" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B78" s="7" t="n">
         <v>19</v>
       </c>
       <c r="C78" s="8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D78" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E78" s="8" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="F78" s="8" t="s">
         <v>25</v>
@@ -5233,35 +5228,35 @@
     </row>
     <row r="79" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="7" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B79" s="7" t="n">
         <v>20</v>
       </c>
       <c r="C79" s="8" t="s">
+        <v>405</v>
+      </c>
+      <c r="D79" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E79" s="8" t="s">
         <v>406</v>
-      </c>
-      <c r="D79" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="E79" s="8" t="s">
-        <v>407</v>
       </c>
       <c r="F79" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G79" s="8" t="s">
+        <v>407</v>
+      </c>
+      <c r="H79" s="8" t="s">
         <v>408</v>
-      </c>
-      <c r="H79" s="8" t="s">
-        <v>409</v>
       </c>
       <c r="I79" s="8"/>
       <c r="J79" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="K79" s="8" t="s">
         <v>410</v>
-      </c>
-      <c r="K79" s="8" t="s">
-        <v>411</v>
       </c>
       <c r="L79" s="9"/>
       <c r="M79" s="10"/>
@@ -5271,31 +5266,31 @@
     </row>
     <row r="80" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="7" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B80" s="7" t="n">
         <v>20</v>
       </c>
       <c r="C80" s="8" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="D80" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E80" s="8" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F80" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G80" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="H80" s="8" t="s">
         <v>414</v>
       </c>
-      <c r="H80" s="8" t="s">
+      <c r="I80" s="8" t="s">
         <v>415</v>
-      </c>
-      <c r="I80" s="8" t="s">
-        <v>416</v>
       </c>
       <c r="J80" s="8"/>
       <c r="K80" s="8"/>
@@ -5307,33 +5302,33 @@
     </row>
     <row r="81" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="7" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B81" s="7" t="n">
         <v>20</v>
       </c>
       <c r="C81" s="8" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="D81" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E81" s="8" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="F81" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G81" s="8" t="s">
+        <v>418</v>
+      </c>
+      <c r="H81" s="8" t="s">
         <v>419</v>
-      </c>
-      <c r="H81" s="8" t="s">
-        <v>420</v>
       </c>
       <c r="I81" s="8"/>
       <c r="J81" s="8"/>
       <c r="K81" s="8" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="L81" s="9"/>
       <c r="M81" s="10"/>
@@ -5343,31 +5338,31 @@
     </row>
     <row r="82" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="7" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B82" s="7" t="n">
         <v>20</v>
       </c>
       <c r="C82" s="8" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="D82" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E82" s="8" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="F82" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G82" s="8" t="s">
+        <v>423</v>
+      </c>
+      <c r="H82" s="8" t="s">
         <v>424</v>
       </c>
-      <c r="H82" s="8" t="s">
+      <c r="I82" s="8" t="s">
         <v>425</v>
-      </c>
-      <c r="I82" s="8" t="s">
-        <v>426</v>
       </c>
       <c r="J82" s="8"/>
       <c r="K82" s="8"/>
@@ -5379,33 +5374,33 @@
     </row>
     <row r="83" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="7" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B83" s="7" t="n">
         <v>20</v>
       </c>
       <c r="C83" s="8" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="D83" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E83" s="8" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F83" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G83" s="8" t="s">
+        <v>428</v>
+      </c>
+      <c r="H83" s="8" t="s">
         <v>429</v>
-      </c>
-      <c r="H83" s="8" t="s">
-        <v>430</v>
       </c>
       <c r="I83" s="8"/>
       <c r="J83" s="8"/>
       <c r="K83" s="8" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="L83" s="9"/>
       <c r="M83" s="10"/>
@@ -5415,37 +5410,37 @@
     </row>
     <row r="84" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="7" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B84" s="7" t="n">
         <v>21</v>
       </c>
       <c r="C84" s="8" t="s">
+        <v>432</v>
+      </c>
+      <c r="D84" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E84" s="8" t="s">
         <v>433</v>
-      </c>
-      <c r="D84" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="E84" s="8" t="s">
-        <v>434</v>
       </c>
       <c r="F84" s="8" t="s">
         <v>23</v>
       </c>
       <c r="G84" s="8" t="s">
+        <v>434</v>
+      </c>
+      <c r="H84" s="8" t="s">
         <v>435</v>
       </c>
-      <c r="H84" s="8" t="s">
+      <c r="I84" s="8" t="s">
         <v>436</v>
       </c>
-      <c r="I84" s="8" t="s">
+      <c r="J84" s="8" t="s">
         <v>437</v>
       </c>
-      <c r="J84" s="8" t="s">
+      <c r="K84" s="8" t="s">
         <v>438</v>
-      </c>
-      <c r="K84" s="8" t="s">
-        <v>439</v>
       </c>
       <c r="L84" s="9"/>
       <c r="M84" s="10"/>
@@ -5455,28 +5450,28 @@
     </row>
     <row r="85" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="7" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B85" s="7" t="n">
         <v>21</v>
       </c>
       <c r="C85" s="8" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="D85" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E85" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F85" s="8" t="s">
         <v>25</v>
       </c>
       <c r="G85" s="8" t="s">
+        <v>441</v>
+      </c>
+      <c r="H85" s="8" t="s">
         <v>442</v>
-      </c>
-      <c r="H85" s="8" t="s">
-        <v>443</v>
       </c>
       <c r="I85" s="8"/>
       <c r="J85" s="8"/>
@@ -5489,31 +5484,31 @@
     </row>
     <row r="86" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="7" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B86" s="7" t="n">
         <v>21</v>
       </c>
       <c r="C86" s="8" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="D86" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E86" s="8" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="F86" s="8" t="s">
         <v>23</v>
       </c>
       <c r="G86" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="H86" s="8" t="s">
         <v>446</v>
       </c>
-      <c r="H86" s="8" t="s">
-        <v>447</v>
-      </c>
       <c r="I86" s="8" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="J86" s="8"/>
       <c r="K86" s="8"/>
@@ -5525,19 +5520,19 @@
     </row>
     <row r="87" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="7" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B87" s="7" t="n">
         <v>22</v>
       </c>
       <c r="C87" s="8" t="s">
+        <v>448</v>
+      </c>
+      <c r="D87" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E87" s="8" t="s">
         <v>449</v>
-      </c>
-      <c r="D87" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="E87" s="8" t="s">
-        <v>450</v>
       </c>
       <c r="F87" s="8" t="s">
         <v>25</v>
@@ -5546,7 +5541,7 @@
         <v>92</v>
       </c>
       <c r="H87" s="8" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="I87" s="8"/>
       <c r="J87" s="8"/>
@@ -5559,35 +5554,35 @@
     </row>
     <row r="88" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="7" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B88" s="7" t="n">
         <v>22</v>
       </c>
       <c r="C88" s="8" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="D88" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E88" s="8" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="F88" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G88" s="8" t="s">
+        <v>453</v>
+      </c>
+      <c r="H88" s="8" t="s">
         <v>454</v>
-      </c>
-      <c r="H88" s="8" t="s">
-        <v>455</v>
       </c>
       <c r="I88" s="8"/>
       <c r="J88" s="8" t="s">
+        <v>455</v>
+      </c>
+      <c r="K88" s="8" t="s">
         <v>456</v>
-      </c>
-      <c r="K88" s="8" t="s">
-        <v>457</v>
       </c>
       <c r="L88" s="9"/>
       <c r="M88" s="10"/>
@@ -5597,33 +5592,33 @@
     </row>
     <row r="89" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="7" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B89" s="7" t="n">
         <v>22</v>
       </c>
       <c r="C89" s="8" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="D89" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E89" s="8" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="F89" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G89" s="8" t="s">
+        <v>459</v>
+      </c>
+      <c r="H89" s="8" t="s">
         <v>460</v>
-      </c>
-      <c r="H89" s="8" t="s">
-        <v>461</v>
       </c>
       <c r="I89" s="8"/>
       <c r="J89" s="8"/>
       <c r="K89" s="8" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="L89" s="9"/>
       <c r="M89" s="10"/>
@@ -5633,31 +5628,31 @@
     </row>
     <row r="90" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="7" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B90" s="7" t="n">
         <v>22</v>
       </c>
       <c r="C90" s="8" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="D90" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E90" s="8" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="F90" s="8" t="s">
         <v>23</v>
       </c>
       <c r="G90" s="8" t="s">
+        <v>464</v>
+      </c>
+      <c r="H90" s="8" t="s">
         <v>465</v>
       </c>
-      <c r="H90" s="8" t="s">
+      <c r="I90" s="8" t="s">
         <v>466</v>
-      </c>
-      <c r="I90" s="8" t="s">
-        <v>467</v>
       </c>
       <c r="J90" s="8"/>
       <c r="K90" s="8"/>
@@ -5669,19 +5664,19 @@
     </row>
     <row r="91" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="7" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B91" s="7" t="n">
         <v>22</v>
       </c>
       <c r="C91" s="8" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="D91" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E91" s="8" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="F91" s="8" t="s">
         <v>25</v>
@@ -5703,28 +5698,28 @@
     </row>
     <row r="92" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="7" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="B92" s="7" t="n">
         <v>23</v>
       </c>
       <c r="C92" s="8" t="s">
+        <v>470</v>
+      </c>
+      <c r="D92" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E92" s="8" t="s">
         <v>471</v>
-      </c>
-      <c r="D92" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="E92" s="8" t="s">
-        <v>472</v>
       </c>
       <c r="F92" s="8" t="s">
         <v>25</v>
       </c>
       <c r="G92" s="8" t="s">
+        <v>472</v>
+      </c>
+      <c r="H92" s="8" t="s">
         <v>473</v>
-      </c>
-      <c r="H92" s="8" t="s">
-        <v>474</v>
       </c>
       <c r="I92" s="8"/>
       <c r="J92" s="8"/>
@@ -5737,28 +5732,28 @@
     </row>
     <row r="93" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="7" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B93" s="7" t="n">
         <v>23</v>
       </c>
       <c r="C93" s="8" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="D93" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E93" s="8" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="F93" s="8" t="s">
         <v>25</v>
       </c>
       <c r="G93" s="8" t="s">
+        <v>476</v>
+      </c>
+      <c r="H93" s="8" t="s">
         <v>477</v>
-      </c>
-      <c r="H93" s="8" t="s">
-        <v>478</v>
       </c>
       <c r="I93" s="8"/>
       <c r="J93" s="8"/>
@@ -5771,28 +5766,28 @@
     </row>
     <row r="94" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="7" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B94" s="7" t="n">
         <v>23</v>
       </c>
       <c r="C94" s="8" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="D94" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E94" s="8" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="F94" s="8" t="s">
         <v>25</v>
       </c>
       <c r="G94" s="8" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="H94" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="I94" s="8"/>
       <c r="J94" s="8"/>
@@ -5805,28 +5800,28 @@
     </row>
     <row r="95" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="7" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B95" s="7" t="n">
         <v>23</v>
       </c>
       <c r="C95" s="8" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="D95" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E95" s="8" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="F95" s="8" t="s">
         <v>25</v>
       </c>
       <c r="G95" s="8" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="H95" s="8" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="I95" s="8"/>
       <c r="J95" s="8"/>
@@ -5839,28 +5834,28 @@
     </row>
     <row r="96" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="7" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B96" s="7" t="n">
         <v>23</v>
       </c>
       <c r="C96" s="8" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="D96" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E96" s="8" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="F96" s="8" t="s">
         <v>25</v>
       </c>
       <c r="G96" s="8" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="H96" s="8" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="I96" s="8"/>
       <c r="J96" s="8"/>
@@ -5873,19 +5868,19 @@
     </row>
     <row r="97" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="7" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B97" s="7" t="n">
         <v>23</v>
       </c>
       <c r="C97" s="8" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="D97" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E97" s="8" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="F97" s="8" t="s">
         <v>25</v>
@@ -5907,33 +5902,33 @@
     </row>
     <row r="98" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="7" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B98" s="7" t="n">
         <v>24</v>
       </c>
       <c r="C98" s="8" t="s">
+        <v>490</v>
+      </c>
+      <c r="D98" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E98" s="8" t="s">
         <v>491</v>
-      </c>
-      <c r="D98" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="E98" s="8" t="s">
-        <v>492</v>
       </c>
       <c r="F98" s="8" t="s">
         <v>23</v>
       </c>
       <c r="G98" s="8" t="s">
+        <v>492</v>
+      </c>
+      <c r="H98" s="8" t="s">
         <v>493</v>
-      </c>
-      <c r="H98" s="8" t="s">
-        <v>494</v>
       </c>
       <c r="I98" s="8"/>
       <c r="J98" s="8"/>
       <c r="K98" s="8" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="L98" s="9"/>
       <c r="M98" s="10"/>
@@ -5943,28 +5938,28 @@
     </row>
     <row r="99" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="7" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B99" s="7" t="n">
         <v>24</v>
       </c>
       <c r="C99" s="8" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="D99" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E99" s="8" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="F99" s="8" t="s">
         <v>23</v>
       </c>
       <c r="G99" s="8" t="s">
+        <v>497</v>
+      </c>
+      <c r="H99" s="8" t="s">
         <v>498</v>
-      </c>
-      <c r="H99" s="8" t="s">
-        <v>499</v>
       </c>
       <c r="I99" s="8"/>
       <c r="J99" s="8"/>
@@ -5979,37 +5974,37 @@
     </row>
     <row r="100" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="7" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="B100" s="7" t="n">
         <v>24</v>
       </c>
       <c r="C100" s="8" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="D100" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E100" s="8" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="F100" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G100" s="8" t="s">
+        <v>501</v>
+      </c>
+      <c r="H100" s="8" t="s">
         <v>502</v>
       </c>
-      <c r="H100" s="8" t="s">
+      <c r="I100" s="8" t="s">
         <v>503</v>
       </c>
-      <c r="I100" s="8" t="s">
+      <c r="J100" s="8" t="s">
         <v>504</v>
       </c>
-      <c r="J100" s="8" t="s">
+      <c r="K100" s="8" t="s">
         <v>505</v>
-      </c>
-      <c r="K100" s="8" t="s">
-        <v>506</v>
       </c>
       <c r="L100" s="9"/>
       <c r="M100" s="10"/>
@@ -6019,34 +6014,34 @@
     </row>
     <row r="101" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="7" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="B101" s="7" t="n">
         <v>24</v>
       </c>
       <c r="C101" s="8" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="D101" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E101" s="8" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="F101" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G101" s="8" t="s">
+        <v>508</v>
+      </c>
+      <c r="H101" s="8" t="s">
         <v>509</v>
       </c>
-      <c r="H101" s="8" t="s">
+      <c r="I101" s="8" t="s">
         <v>510</v>
       </c>
-      <c r="I101" s="8" t="s">
+      <c r="J101" s="8" t="s">
         <v>511</v>
-      </c>
-      <c r="J101" s="8" t="s">
-        <v>512</v>
       </c>
       <c r="K101" s="8" t="s">
         <v>73</v>
@@ -6059,33 +6054,33 @@
     </row>
     <row r="102" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="7" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B102" s="7" t="n">
         <v>24</v>
       </c>
       <c r="C102" s="8" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="D102" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E102" s="8" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="F102" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G102" s="8" t="s">
+        <v>514</v>
+      </c>
+      <c r="H102" s="8" t="s">
         <v>515</v>
-      </c>
-      <c r="H102" s="8" t="s">
-        <v>516</v>
       </c>
       <c r="I102" s="8"/>
       <c r="J102" s="8"/>
       <c r="K102" s="8" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="L102" s="9"/>
       <c r="M102" s="10"/>
@@ -6095,19 +6090,19 @@
     </row>
     <row r="103" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="7" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="B103" s="7" t="n">
         <v>24</v>
       </c>
       <c r="C103" s="8" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="D103" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E103" s="8" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="F103" s="8" t="s">
         <v>25</v>
@@ -6116,7 +6111,7 @@
         <v>92</v>
       </c>
       <c r="H103" s="8" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="I103" s="8"/>
       <c r="J103" s="8"/>
@@ -6129,19 +6124,19 @@
     </row>
     <row r="104" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="7" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B104" s="7" t="n">
         <v>25</v>
       </c>
       <c r="C104" s="8" t="s">
+        <v>521</v>
+      </c>
+      <c r="D104" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E104" s="8" t="s">
         <v>522</v>
-      </c>
-      <c r="D104" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="E104" s="8" t="s">
-        <v>523</v>
       </c>
       <c r="F104" s="8" t="s">
         <v>25</v>
@@ -6150,7 +6145,7 @@
         <v>92</v>
       </c>
       <c r="H104" s="8" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="I104" s="8"/>
       <c r="J104" s="8"/>
@@ -6163,19 +6158,19 @@
     </row>
     <row r="105" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="7" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="B105" s="7" t="n">
         <v>25</v>
       </c>
       <c r="C105" s="8" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="D105" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E105" s="8" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="F105" s="8" t="s">
         <v>25</v>
@@ -6184,7 +6179,7 @@
         <v>92</v>
       </c>
       <c r="H105" s="8" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="I105" s="8"/>
       <c r="J105" s="8"/>
@@ -6197,19 +6192,19 @@
     </row>
     <row r="106" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="7" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="B106" s="7" t="n">
         <v>25</v>
       </c>
       <c r="C106" s="8" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="D106" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E106" s="8" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="F106" s="8" t="s">
         <v>25</v>
@@ -6218,7 +6213,7 @@
         <v>92</v>
       </c>
       <c r="H106" s="8" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="I106" s="8"/>
       <c r="J106" s="8"/>
@@ -6231,19 +6226,19 @@
     </row>
     <row r="107" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="7" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B107" s="7" t="n">
         <v>25</v>
       </c>
       <c r="C107" s="8" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="D107" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E107" s="8" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="F107" s="8" t="s">
         <v>25</v>
@@ -6252,7 +6247,7 @@
         <v>92</v>
       </c>
       <c r="H107" s="8" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="I107" s="8"/>
       <c r="J107" s="8"/>
@@ -6265,31 +6260,31 @@
     </row>
     <row r="108" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B108" s="7" t="n">
         <v>25</v>
       </c>
       <c r="C108" s="8" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="D108" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E108" s="8" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="F108" s="8" t="s">
         <v>23</v>
       </c>
       <c r="G108" s="8" t="s">
+        <v>535</v>
+      </c>
+      <c r="H108" s="8" t="s">
         <v>536</v>
       </c>
-      <c r="H108" s="8" t="s">
+      <c r="I108" s="8" t="s">
         <v>537</v>
-      </c>
-      <c r="I108" s="8" t="s">
-        <v>538</v>
       </c>
       <c r="J108" s="8"/>
       <c r="K108" s="8"/>
@@ -6301,34 +6296,34 @@
     </row>
     <row r="109" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="7" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="B109" s="7" t="n">
         <v>25</v>
       </c>
       <c r="C109" s="8" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="D109" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E109" s="8" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="F109" s="8" t="s">
         <v>23</v>
       </c>
       <c r="G109" s="8" t="s">
+        <v>540</v>
+      </c>
+      <c r="H109" s="8" t="s">
         <v>541</v>
-      </c>
-      <c r="H109" s="8" t="s">
-        <v>542</v>
       </c>
       <c r="I109" s="8" t="s">
         <v>222</v>
       </c>
       <c r="J109" s="8" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="K109" s="8"/>
       <c r="L109" s="9"/>
@@ -6339,28 +6334,28 @@
     </row>
     <row r="110" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="7" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B110" s="7" t="n">
         <v>25</v>
       </c>
       <c r="C110" s="8" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="D110" s="8" t="s">
         <v>45</v>
       </c>
       <c r="E110" s="8" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="F110" s="8" t="s">
         <v>25</v>
       </c>
       <c r="G110" s="8" t="s">
+        <v>545</v>
+      </c>
+      <c r="H110" s="8" t="s">
         <v>546</v>
-      </c>
-      <c r="H110" s="8" t="s">
-        <v>547</v>
       </c>
       <c r="I110" s="8"/>
       <c r="J110" s="8"/>
@@ -6373,19 +6368,19 @@
     </row>
     <row r="111" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="7" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B111" s="7" t="n">
         <v>25</v>
       </c>
       <c r="C111" s="8" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="D111" s="8" t="s">
         <v>75</v>
       </c>
       <c r="E111" s="8" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="F111" s="8" t="s">
         <v>25</v>
@@ -6394,7 +6389,7 @@
         <v>92</v>
       </c>
       <c r="H111" s="8" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="I111" s="8"/>
       <c r="J111" s="8"/>
@@ -6407,19 +6402,19 @@
     </row>
     <row r="112" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="7" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="B112" s="7" t="n">
         <v>25</v>
       </c>
       <c r="C112" s="8" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="D112" s="8" t="s">
         <v>75</v>
       </c>
       <c r="E112" s="8" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="F112" s="8" t="s">
         <v>25</v>
@@ -6484,22 +6479,22 @@
         <v>31</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>552</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>553</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="E1" s="6" t="s">
         <v>554</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>555</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>556</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>557</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>558</v>
       </c>
       <c r="I1" s="6" t="s">
         <v>18</v>
@@ -6870,7 +6865,7 @@
         <v>14</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C12" s="7" t="n">
         <f aca="false">COUNTIF(Checklist!$B$2:$B$112,A12)</f>
@@ -6906,7 +6901,7 @@
         <v>15</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C13" s="7" t="n">
         <f aca="false">COUNTIF(Checklist!$B$2:$B$112,A13)</f>
@@ -6942,7 +6937,7 @@
         <v>16</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C14" s="7" t="n">
         <f aca="false">COUNTIF(Checklist!$B$2:$B$112,A14)</f>
@@ -6978,7 +6973,7 @@
         <v>17</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C15" s="7" t="n">
         <f aca="false">COUNTIF(Checklist!$B$2:$B$112,A15)</f>
@@ -7014,7 +7009,7 @@
         <v>18</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C16" s="7" t="n">
         <f aca="false">COUNTIF(Checklist!$B$2:$B$112,A16)</f>
@@ -7050,7 +7045,7 @@
         <v>19</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C17" s="7" t="n">
         <f aca="false">COUNTIF(Checklist!$B$2:$B$112,A17)</f>
@@ -7086,7 +7081,7 @@
         <v>20</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C18" s="7" t="n">
         <f aca="false">COUNTIF(Checklist!$B$2:$B$112,A18)</f>
@@ -7122,7 +7117,7 @@
         <v>21</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="C19" s="7" t="n">
         <f aca="false">COUNTIF(Checklist!$B$2:$B$112,A19)</f>
@@ -7158,7 +7153,7 @@
         <v>22</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="C20" s="7" t="n">
         <f aca="false">COUNTIF(Checklist!$B$2:$B$112,A20)</f>
@@ -7194,7 +7189,7 @@
         <v>23</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="C21" s="7" t="n">
         <f aca="false">COUNTIF(Checklist!$B$2:$B$112,A21)</f>
@@ -7230,7 +7225,7 @@
         <v>24</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C22" s="7" t="n">
         <f aca="false">COUNTIF(Checklist!$B$2:$B$112,A22)</f>
@@ -7266,7 +7261,7 @@
         <v>25</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="C23" s="7" t="n">
         <f aca="false">COUNTIF(Checklist!$B$2:$B$112,A23)</f>
@@ -7300,7 +7295,7 @@
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13"/>
       <c r="B24" s="14" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="C24" s="13" t="n">
         <f aca="false">SUM(C2:C23)</f>

</xml_diff>